<commit_message>
Version base datos prueba
</commit_message>
<xml_diff>
--- a/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-08.xlsx
+++ b/Documents/caapd-facturacion/escritorio/Base de datos/PADRON_MES_2026-08.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15 06:26:17</t>
+          <t>2026-10-15 07:07:03</t>
         </is>
       </c>
     </row>
@@ -6658,7 +6658,7 @@
     "fecha_emision": "2026-08-26",
     "fecha_vencimiento": "2026-09-10"
   },
-  "ultimo_envio_lectores": "2026-10-15 06:26:16"
+  "ultimo_envio_lectores": "2026-10-15 07:07:03"
 }</t>
         </is>
       </c>

</xml_diff>